<commit_message>
imrpoved a wee bit.
</commit_message>
<xml_diff>
--- a/docs/relay/design/scripting.xlsx
+++ b/docs/relay/design/scripting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\js\games\docs\relay\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3285935D-95CF-4AD5-B1FE-40AB32625A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC73DFB3-A9CD-4EE6-A081-DCF47947ECC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
   <si>
     <t>firstletter</t>
   </si>
@@ -329,7 +329,39 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1565,10 +1597,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:AB2">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C31">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
works wonderfully, both at 20hz and 5hz
</commit_message>
<xml_diff>
--- a/docs/relay/design/scripting.xlsx
+++ b/docs/relay/design/scripting.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\js\games\docs\relay\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_B4816EE8B5370BE58DA68AD559D404E83482B4A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12580"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheetwithani" sheetId="3" r:id="rId1"/>
     <sheet name="conventions" sheetId="4" r:id="rId2"/>
     <sheet name="bad" sheetId="1" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,14 +38,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -436,7 +437,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -520,7 +521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -529,249 +530,31 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="28">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -853,6 +636,51 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1131,38 +959,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.90625" customWidth="1"/>
-    <col min="2" max="2" width="4.08984375" customWidth="1"/>
+    <col min="1" max="1" width="1.88671875" customWidth="1"/>
+    <col min="2" max="2" width="4.109375" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="5.1796875" style="14" customWidth="1"/>
-    <col min="5" max="5" width="7" style="14" customWidth="1"/>
-    <col min="6" max="6" width="20.36328125" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" customWidth="1"/>
-    <col min="8" max="15" width="7.08984375" customWidth="1"/>
-    <col min="16" max="16" width="30.81640625" customWidth="1"/>
-    <col min="17" max="17" width="15.1796875" customWidth="1"/>
-    <col min="18" max="18" width="12.1796875" customWidth="1"/>
-    <col min="19" max="19" width="15.1796875" customWidth="1"/>
-    <col min="20" max="20" width="15.36328125" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" customWidth="1"/>
+    <col min="8" max="15" width="7.109375" customWidth="1"/>
+    <col min="16" max="16" width="30.77734375" customWidth="1"/>
+    <col min="17" max="17" width="15.21875" customWidth="1"/>
+    <col min="18" max="18" width="12.21875" customWidth="1"/>
+    <col min="19" max="19" width="15.21875" customWidth="1"/>
+    <col min="20" max="20" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="H1" s="8" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H1" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8" t="s">
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
       <c r="P1" t="s">
         <v>94</v>
       </c>
@@ -1173,7 +1001,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="C2" t="s">
         <v>119</v>
       </c>
@@ -1213,17 +1041,17 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" t="s">
         <v>111</v>
       </c>
       <c r="F3" t="s">
@@ -1264,7 +1092,7 @@
         <v>['terminal','delay','bucket','pretty','action','energy','water','food','parts','antimatter','coolant','minerals','salvage','description'],</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>65</v>
       </c>
@@ -1275,10 +1103,10 @@
       <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4">
         <v>15</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" s="4" t="s">
@@ -1299,7 +1127,7 @@
         <v>['reactor',15,0,'Reactor','REPAIR',50,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="12"/>
       <c r="B5">
         <f t="shared" ref="B5:B44" si="2">SUM(H5:O5)</f>
@@ -1308,10 +1136,10 @@
       <c r="C5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5">
         <v>8</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5">
         <v>10</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -1335,7 +1163,7 @@
         <v>['solar',8,10,'Solar Array','REPAIR',30,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="12"/>
       <c r="B6">
         <f t="shared" si="2"/>
@@ -1344,10 +1172,10 @@
       <c r="C6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6">
         <v>12</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6">
         <v>0</v>
       </c>
       <c r="F6" s="4" t="s">
@@ -1371,7 +1199,7 @@
         <v>['life',12,0,'Life Support','REPAIR',0,20,20,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="12"/>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -1380,10 +1208,10 @@
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7">
         <v>6</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7">
         <v>10</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -1407,7 +1235,7 @@
         <v>['water',6,10,'Water Recycler','REPAIR',0,30,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="12"/>
       <c r="B8">
         <f t="shared" si="2"/>
@@ -1416,10 +1244,10 @@
       <c r="C8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8">
         <v>13</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8">
         <v>10</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -1443,7 +1271,7 @@
         <v>['hydro',13,10,'Hydroponics','REPAIR',0,0,30,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9">
         <f t="shared" si="2"/>
@@ -1452,10 +1280,10 @@
       <c r="C9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9">
         <v>4</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9">
         <v>0</v>
       </c>
       <c r="F9" s="4" t="s">
@@ -1476,7 +1304,7 @@
         <v>['cargo',4,0,'Cargo bay','REPAIR',0,0,0,20,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10">
         <f t="shared" si="2"/>
@@ -1485,10 +1313,10 @@
       <c r="C10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10">
         <v>11</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10">
         <v>10</v>
       </c>
       <c r="F10" s="5" t="s">
@@ -1512,7 +1340,7 @@
         <v>['comms',11,10,'Comms array','REPAIR',0,0,0,50,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="12"/>
       <c r="B11">
         <f t="shared" si="2"/>
@@ -1521,10 +1349,10 @@
       <c r="C11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11">
         <v>13</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11">
         <v>20</v>
       </c>
       <c r="F11" s="6" t="s">
@@ -1548,7 +1376,7 @@
         <v>['fab',13,20,'Fabricator','REPAIR',0,0,0,10,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12">
         <f t="shared" si="2"/>
@@ -1557,10 +1385,10 @@
       <c r="C12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12">
         <v>14</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12">
         <v>20</v>
       </c>
       <c r="F12" s="6" t="s">
@@ -1587,7 +1415,7 @@
         <v>['med',14,20,'Medical bay','REPAIR',0,10,10,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13">
         <f t="shared" si="2"/>
@@ -1596,10 +1424,10 @@
       <c r="C13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13">
         <v>20</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13">
         <v>20</v>
       </c>
       <c r="F13" s="6" t="s">
@@ -1626,8 +1454,8 @@
         <v>['anti',20,20,'Antimatter Chamber','REPAIR',10,0,0,0,5,0,0,0,0],</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
+    <row r="14" spans="1:20" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15" t="s">
         <v>66</v>
       </c>
       <c r="B14">
@@ -1637,7 +1465,7 @@
       <c r="C14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14">
         <v>30</v>
       </c>
       <c r="F14" s="7" t="s">
@@ -1660,8 +1488,8 @@
         <v>['hazard',0,30,'Space Hazard Unit','REPAIR',0,0,0,0,0,0,0,0,'Allows you to explore space.'],</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A15" s="11"/>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A15" s="15"/>
       <c r="B15">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -1669,23 +1497,23 @@
       <c r="C15" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="P15" s="9" t="s">
+      <c r="P15" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="Q15" s="9"/>
+      <c r="Q15" s="8"/>
       <c r="T15" t="str">
         <f t="shared" si="1"/>
         <v>['obs',0,0,'Observatory','WORLDMAP',0,0,0,0,0,0,0,0,'Lets you peek into the endless void of space.'],</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="11"/>
+    <row r="16" spans="1:20" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15"/>
       <c r="B16">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -1693,14 +1521,14 @@
       <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
       <c r="R16" t="s">
         <v>81</v>
       </c>
@@ -1709,8 +1537,8 @@
         <v>['shuttle',0,0,'Shuttle bay','TRAVEL',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A17" s="11"/>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
       <c r="B17">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -1718,21 +1546,21 @@
       <c r="C17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="P17" s="9"/>
-      <c r="Q17" s="9"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
       <c r="T17" t="str">
         <f t="shared" si="1"/>
         <v>['upgrade',0,0,'Upgrade center','SEEUPGRADES',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
         <v>67</v>
       </c>
       <c r="B18">
@@ -1742,10 +1570,10 @@
       <c r="C18" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18">
         <v>5</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E18">
         <v>30</v>
       </c>
       <c r="F18" s="3" t="s">
@@ -1764,8 +1592,8 @@
         <v>['mining',5,30,'Mining station','CAPTURE',0,0,0,0,0,0,15,0,0],</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A19" s="10"/>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A19" s="14"/>
       <c r="B19">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -1773,10 +1601,10 @@
       <c r="C19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19">
         <v>5</v>
       </c>
-      <c r="E19" s="14">
+      <c r="E19">
         <v>30</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -1795,8 +1623,8 @@
         <v>['scrapyard',5,30,'Scrapyard','CAPTURE',0,0,0,0,0,0,0,15,0],</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A20" s="10"/>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A20" s="14"/>
       <c r="B20">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -1804,10 +1632,10 @@
       <c r="C20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20">
         <v>5</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20">
         <v>30</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -1832,8 +1660,8 @@
         <v>['data',5,30,'Data vault','CAPTURE',0,0,0,0,0,5,5,5,0],</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A21" s="10"/>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A21" s="14"/>
       <c r="B21">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -1841,10 +1669,10 @@
       <c r="C21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21">
         <v>5</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21">
         <v>30</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -1860,8 +1688,8 @@
         <v>['supply',5,30,'Supply depot','CAPTURE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A22" s="10"/>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A22" s="14"/>
       <c r="B22">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -1869,10 +1697,10 @@
       <c r="C22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22">
         <v>5</v>
       </c>
-      <c r="E22" s="14">
+      <c r="E22">
         <v>40</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -1891,8 +1719,8 @@
         <v>['fusion',5,40,'Fusion core','CAPTURE',0,0,0,0,15,0,0,0,0],</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A23" s="10"/>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="14"/>
       <c r="B23">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -1900,10 +1728,10 @@
       <c r="C23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23">
         <v>5</v>
       </c>
-      <c r="E23" s="14">
+      <c r="E23">
         <v>30</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -1925,8 +1753,8 @@
         <v>['alloy',5,30,'Alloy plant','CAPTURE',0,0,0,0,0,0,10,5,0],</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A24" s="10"/>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A24" s="14"/>
       <c r="B24">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -1934,10 +1762,10 @@
       <c r="C24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24">
         <v>5</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24">
         <v>40</v>
       </c>
       <c r="F24" s="3" t="s">
@@ -1962,8 +1790,8 @@
         <v>['research',5,40,'Research lab','CAPTURE',0,0,0,0,5,5,0,5,0],</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A25" s="10"/>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A25" s="14"/>
       <c r="B25">
         <f t="shared" si="2"/>
         <v>120</v>
@@ -1971,7 +1799,7 @@
       <c r="C25" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E25" s="14">
+      <c r="E25">
         <v>20</v>
       </c>
       <c r="F25" s="3" t="s">
@@ -1986,8 +1814,8 @@
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A26" s="10"/>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A26" s="14"/>
       <c r="B26">
         <f t="shared" si="2"/>
         <v>120</v>
@@ -1995,7 +1823,7 @@
       <c r="C26" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="14">
+      <c r="E26">
         <v>20</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -2010,8 +1838,8 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A27" s="10"/>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A27" s="14"/>
       <c r="B27">
         <f t="shared" si="2"/>
         <v>120</v>
@@ -2019,7 +1847,7 @@
       <c r="C27" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27">
         <v>20</v>
       </c>
       <c r="F27" s="3" t="s">
@@ -2034,8 +1862,8 @@
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A28" s="10"/>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A28" s="14"/>
       <c r="B28">
         <f t="shared" si="2"/>
         <v>120</v>
@@ -2043,7 +1871,7 @@
       <c r="C28" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E28" s="14">
+      <c r="E28">
         <v>20</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -2058,8 +1886,8 @@
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A29" s="10"/>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="14"/>
       <c r="B29">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2067,7 +1895,7 @@
       <c r="C29" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E29" s="14">
+      <c r="E29">
         <v>40</v>
       </c>
       <c r="F29" s="3" t="s">
@@ -2086,8 +1914,8 @@
         <v>['chestantimatter',0,40,'Antimatter traces','CLAIM',0,0,0,0,80,0,0,0,0],</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A30" s="10"/>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A30" s="14"/>
       <c r="B30">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2095,7 +1923,7 @@
       <c r="C30" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E30" s="14">
+      <c r="E30">
         <v>40</v>
       </c>
       <c r="F30" s="3" t="s">
@@ -2114,8 +1942,8 @@
         <v>['chestcoolant',0,40,'Coolant remains','CLAIM',0,0,0,0,0,80,0,0,0],</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A31" s="10"/>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A31" s="14"/>
       <c r="B31">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2123,7 +1951,7 @@
       <c r="C31" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E31" s="14">
+      <c r="E31">
         <v>40</v>
       </c>
       <c r="F31" s="3" t="s">
@@ -2142,8 +1970,8 @@
         <v>['chestmineral',0,40,'Mineral residue','CLAIM',0,0,0,0,0,0,80,0,0],</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A32" s="10"/>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A32" s="14"/>
       <c r="B32">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2151,7 +1979,7 @@
       <c r="C32" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E32" s="14">
+      <c r="E32">
         <v>40</v>
       </c>
       <c r="F32" s="3" t="s">
@@ -2170,8 +1998,8 @@
         <v>['chestsalvage',0,40,'Salvage pack','CLAIM',0,0,0,0,0,0,0,80,0],</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A33" s="10"/>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A33" s="14"/>
       <c r="B33">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -2179,7 +2007,7 @@
       <c r="C33" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E33" s="14">
+      <c r="E33">
         <v>0</v>
       </c>
       <c r="F33" s="3" t="s">
@@ -2195,8 +2023,8 @@
         <v>['door_easy',0,0,'Damaged door','HACK',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A34" s="10"/>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A34" s="14"/>
       <c r="B34">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -2204,7 +2032,7 @@
       <c r="C34" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E34" s="14">
+      <c r="E34">
         <v>20</v>
       </c>
       <c r="F34" s="3" t="s">
@@ -2220,8 +2048,8 @@
         <v>['door_medium',0,20,'Locked door','HACK',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A35" s="10"/>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A35" s="14"/>
       <c r="B35">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -2229,7 +2057,7 @@
       <c r="C35" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E35" s="14">
+      <c r="E35">
         <v>50</v>
       </c>
       <c r="F35" s="3" t="s">
@@ -2245,8 +2073,8 @@
         <v>['door_hard',0,50,'High security door','HACK',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A36" s="10"/>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A36" s="14"/>
       <c r="B36">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -2260,7 +2088,7 @@
         <v>[0,0,0,0,0,0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>95</v>
       </c>
@@ -2268,153 +2096,153 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E37" s="14">
+      <c r="E37">
         <v>10</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="9" t="s">
         <v>98</v>
       </c>
       <c r="G37" t="s">
         <v>108</v>
       </c>
-      <c r="P37" s="13"/>
-      <c r="Q37" s="13"/>
+      <c r="P37" s="9"/>
+      <c r="Q37" s="9"/>
       <c r="T37" t="str">
         <f t="shared" si="1"/>
         <v>['plants',0,10,'Plants','RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="12"/>
       <c r="B38">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="E38" s="14">
+      <c r="E38">
         <v>10</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F38" s="9" t="s">
         <v>110</v>
       </c>
       <c r="G38" t="s">
         <v>108</v>
       </c>
-      <c r="P38" s="13"/>
-      <c r="Q38" s="13"/>
+      <c r="P38" s="9"/>
+      <c r="Q38" s="9"/>
       <c r="T38" t="str">
         <f t="shared" si="1"/>
         <v>['fridge',0,10,'Fridge','RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="12"/>
       <c r="B39">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C39" s="13"/>
-      <c r="F39" s="13"/>
+      <c r="C39" s="9"/>
+      <c r="F39" s="9"/>
       <c r="G39" t="s">
         <v>108</v>
       </c>
-      <c r="P39" s="13"/>
-      <c r="Q39" s="13"/>
+      <c r="P39" s="9"/>
+      <c r="Q39" s="9"/>
       <c r="T39" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="12"/>
       <c r="B40">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C40" s="13"/>
-      <c r="F40" s="13"/>
+      <c r="C40" s="9"/>
+      <c r="F40" s="9"/>
       <c r="G40" t="s">
         <v>108</v>
       </c>
-      <c r="P40" s="13"/>
-      <c r="Q40" s="13"/>
+      <c r="P40" s="9"/>
+      <c r="Q40" s="9"/>
       <c r="T40" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="12"/>
       <c r="B41">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C41" s="13"/>
-      <c r="F41" s="13"/>
+      <c r="C41" s="9"/>
+      <c r="F41" s="9"/>
       <c r="G41" t="s">
         <v>108</v>
       </c>
-      <c r="P41" s="13"/>
-      <c r="Q41" s="13"/>
+      <c r="P41" s="9"/>
+      <c r="Q41" s="9"/>
       <c r="T41" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="12"/>
       <c r="B42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C42" s="13"/>
-      <c r="F42" s="13"/>
+      <c r="C42" s="9"/>
+      <c r="F42" s="9"/>
       <c r="G42" t="s">
         <v>108</v>
       </c>
-      <c r="P42" s="13"/>
-      <c r="Q42" s="13"/>
+      <c r="P42" s="9"/>
+      <c r="Q42" s="9"/>
       <c r="T42" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="12"/>
       <c r="B43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C43" s="13"/>
-      <c r="F43" s="13"/>
+      <c r="C43" s="9"/>
+      <c r="F43" s="9"/>
       <c r="G43" t="s">
         <v>108</v>
       </c>
-      <c r="P43" s="13"/>
-      <c r="Q43" s="13"/>
+      <c r="P43" s="9"/>
+      <c r="Q43" s="9"/>
       <c r="T43" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="12"/>
       <c r="B44">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C44" s="13"/>
-      <c r="F44" s="13"/>
+      <c r="C44" s="9"/>
+      <c r="F44" s="9"/>
       <c r="G44" t="s">
         <v>108</v>
       </c>
-      <c r="P44" s="13"/>
-      <c r="Q44" s="13"/>
+      <c r="P44" s="9"/>
+      <c r="Q44" s="9"/>
       <c r="T44" t="str">
         <f t="shared" si="1"/>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
@@ -2429,29 +2257,14 @@
     <mergeCell ref="L1:O1"/>
     <mergeCell ref="A14:A17"/>
   </mergeCells>
+  <conditionalFormatting sqref="C1:C17 C37:C1048576">
+    <cfRule type="duplicateValues" dxfId="11" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="10" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D2:O2 T2:U2">
-    <cfRule type="duplicateValues" dxfId="16" priority="15"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:S2">
-    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q3:R3">
-    <cfRule type="duplicateValues" dxfId="14" priority="9"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C17 C37:C1048576">
-    <cfRule type="duplicateValues" dxfId="13" priority="16"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2">
-    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P3">
-    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P37:Q44">
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F37:F44">
-    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E4:E62">
     <cfRule type="colorScale" priority="2">
@@ -2465,8 +2278,23 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="F37:F44">
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2">
+    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P37:Q44">
+    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q3:R3">
+    <cfRule type="duplicateValues" dxfId="4" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:S2">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2474,20 +2302,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="97.453125" defaultRowHeight="57" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="97.44140625" defaultRowHeight="57" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="97.453125" style="15"/>
+    <col min="1" max="16384" width="97.44140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2497,17 +2325,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:Z31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="6" width="7.36328125" customWidth="1"/>
-    <col min="7" max="7" width="14.36328125" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" customWidth="1"/>
+    <col min="5" max="6" width="7.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:26" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
         <v>0</v>
       </c>
@@ -2579,7 +2407,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -2622,15 +2450,15 @@
       <c r="O3" t="s">
         <v>11</v>
       </c>
-      <c r="P3" t="e" cm="1">
-        <f t="array" aca="1" ref="P3" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D3:O3),""""&amp;D3:O3&amp;"""",IF(D3:O3="",0,D3:O3)))&amp;"],"</f>
-        <v>#NAME?</v>
-      </c>
-    </row>
-    <row r="4" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B4" t="e">
-        <f ca="1">SUM(E4:AA4)</f>
-        <v>#NAME?</v>
+      <c r="P3" t="str" cm="1">
+        <f t="array" ref="P3">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D3:O3),""""&amp;D3:O3&amp;"""",IF(D3:O3="",0,D3:O3)))&amp;"],"</f>
+        <v>["terminal","delay","question","pretty","action","energy","food","water","parts","metals","titanium","alloy"],</v>
+      </c>
+    </row>
+    <row r="4" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <f>SUM(E4:AA4)</f>
+        <v>55</v>
       </c>
       <c r="C4" t="str">
         <f>LEFT(D4,1)</f>
@@ -2654,15 +2482,15 @@
       <c r="I4">
         <v>40</v>
       </c>
-      <c r="P4" t="e" cm="1">
-        <f t="array" aca="1" ref="P4" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D4:O4),""""&amp;D4:O4&amp;"""",IF(D4:O4="",0,D4:O4)))&amp;"],"</f>
-        <v>#NAME?</v>
-      </c>
-    </row>
-    <row r="5" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B5" t="e">
-        <f t="shared" ref="B5:B31" ca="1" si="1">SUM(E5:AA5)</f>
-        <v>#NAME?</v>
+      <c r="P4" t="str" cm="1">
+        <f t="array" ref="P4">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D4:O4),""""&amp;D4:O4&amp;"""",IF(D4:O4="",0,D4:O4)))&amp;"],"</f>
+        <v>["reactor",15,0,"Reactor","REPAIR",40,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="5" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <f t="shared" ref="B5:B31" si="1">SUM(E5:AA5)</f>
+        <v>55</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" ref="C5:C31" si="2">LEFT(D5,1)</f>
@@ -2686,19 +2514,19 @@
       <c r="I5">
         <v>25</v>
       </c>
-      <c r="P5" t="e" cm="1">
-        <f t="array" aca="1" ref="P5" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D5:O5),""""&amp;D5:O5&amp;"""",IF(D5:O5="",0,D5:O5)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P5" t="str" cm="1">
+        <f t="array" ref="P5">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D5:O5),""""&amp;D5:O5&amp;"""",IF(D5:O5="",0,D5:O5)))&amp;"],"</f>
+        <v>["solar",20,10,"Solar Array","REPAIR",25,0,0,0,0,0,0],</v>
       </c>
       <c r="S5" t="str">
         <f>" * @property {number} "&amp;D5</f>
         <v xml:space="preserve"> * @property {number} solar</v>
       </c>
     </row>
-    <row r="6" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B6" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="6" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <f t="shared" si="1"/>
+        <v>57</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="2"/>
@@ -2725,19 +2553,19 @@
       <c r="K6">
         <v>10</v>
       </c>
-      <c r="P6" t="e" cm="1">
-        <f t="array" aca="1" ref="P6" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D6:O6),""""&amp;D6:O6&amp;"""",IF(D6:O6="",0,D6:O6)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P6" t="str" cm="1">
+        <f t="array" ref="P6">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D6:O6),""""&amp;D6:O6&amp;"""",IF(D6:O6="",0,D6:O6)))&amp;"],"</f>
+        <v>["hydro",12,20,"Hydroponics","REPAIR",0,15,10,0,0,0,0],</v>
       </c>
       <c r="S6" t="str">
         <f t="shared" ref="S6:S23" si="3">" * @property {number} "&amp;D6</f>
         <v xml:space="preserve"> * @property {number} hydro</v>
       </c>
     </row>
-    <row r="7" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B7" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="7" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <f t="shared" si="1"/>
+        <v>55</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="2"/>
@@ -2761,19 +2589,19 @@
       <c r="K7">
         <v>25</v>
       </c>
-      <c r="P7" t="e" cm="1">
-        <f t="array" aca="1" ref="P7" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D7:O7),""""&amp;D7:O7&amp;"""",IF(D7:O7="",0,D7:O7)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P7" t="str" cm="1">
+        <f t="array" ref="P7">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D7:O7),""""&amp;D7:O7&amp;"""",IF(D7:O7="",0,D7:O7)))&amp;"],"</f>
+        <v>["water",10,20,"Water recycler","REPAIR",0,0,25,0,0,0,0],</v>
       </c>
       <c r="S7" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} water</v>
       </c>
     </row>
-    <row r="8" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="8" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <f t="shared" si="1"/>
+        <v>48</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="2"/>
@@ -2800,19 +2628,19 @@
       <c r="L8">
         <v>10</v>
       </c>
-      <c r="P8" t="e" cm="1">
-        <f t="array" aca="1" ref="P8" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D8:O8),""""&amp;D8:O8&amp;"""",IF(D8:O8="",0,D8:O8)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P8" t="str" cm="1">
+        <f t="array" ref="P8">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D8:O8),""""&amp;D8:O8&amp;"""",IF(D8:O8="",0,D8:O8)))&amp;"],"</f>
+        <v>["cargo",8,20,"Cargo bay","REPAIR",0,10,0,10,0,0,0],</v>
       </c>
       <c r="S8" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} cargo</v>
       </c>
     </row>
-    <row r="9" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B9" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="9" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <f t="shared" si="1"/>
+        <v>92</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="2"/>
@@ -2836,19 +2664,19 @@
       <c r="L9">
         <v>30</v>
       </c>
-      <c r="P9" t="e" cm="1">
-        <f t="array" aca="1" ref="P9" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D9:O9),""""&amp;D9:O9&amp;"""",IF(D9:O9="",0,D9:O9)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P9" t="str" cm="1">
+        <f t="array" ref="P9">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D9:O9),""""&amp;D9:O9&amp;"""",IF(D9:O9="",0,D9:O9)))&amp;"],"</f>
+        <v>["comms",12,50,"Comms array","REPAIR",0,0,0,30,0,0,0],</v>
       </c>
       <c r="S9" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} comms</v>
       </c>
     </row>
-    <row r="10" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B10" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="10" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <f t="shared" si="1"/>
+        <v>95</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="2"/>
@@ -2875,19 +2703,19 @@
       <c r="L10">
         <v>5</v>
       </c>
-      <c r="P10" t="e" cm="1">
-        <f t="array" aca="1" ref="P10" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D10:O10),""""&amp;D10:O10&amp;"""",IF(D10:O10="",0,D10:O10)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P10" t="str" cm="1">
+        <f t="array" ref="P10">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D10:O10),""""&amp;D10:O10&amp;"""",IF(D10:O10="",0,D10:O10)))&amp;"],"</f>
+        <v>["fab",10,60,"Fabricator","REPAIR",0,0,20,5,0,0,0],</v>
       </c>
       <c r="S10" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} fab</v>
       </c>
     </row>
-    <row r="11" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B11" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="11" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <f t="shared" si="1"/>
+        <v>50</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="2"/>
@@ -2911,19 +2739,19 @@
       <c r="L11">
         <v>10</v>
       </c>
-      <c r="P11" t="e" cm="1">
-        <f t="array" aca="1" ref="P11" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D11:O11),""""&amp;D11:O11&amp;"""",IF(D11:O11="",0,D11:O11)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P11" t="str" cm="1">
+        <f t="array" ref="P11">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D11:O11),""""&amp;D11:O11&amp;"""",IF(D11:O11="",0,D11:O11)))&amp;"],"</f>
+        <v>["med",10,30,"Medical bay","REPAIR",0,0,0,10,0,0,0],</v>
       </c>
       <c r="S11" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} med</v>
       </c>
     </row>
-    <row r="12" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B12" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="12" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <f t="shared" si="1"/>
+        <v>55</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="2"/>
@@ -2950,19 +2778,19 @@
       <c r="K12">
         <v>15</v>
       </c>
-      <c r="P12" t="e" cm="1">
-        <f t="array" aca="1" ref="P12" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D12:O12),""""&amp;D12:O12&amp;"""",IF(D12:O12="",0,D12:O12)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P12" t="str" cm="1">
+        <f t="array" ref="P12">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D12:O12),""""&amp;D12:O12&amp;"""",IF(D12:O12="",0,D12:O12)))&amp;"],"</f>
+        <v>["life",20,10,"Life support","REPAIR",0,10,15,0,0,0,0],</v>
       </c>
       <c r="S12" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} life</v>
       </c>
     </row>
-    <row r="13" spans="2:26" x14ac:dyDescent="0.35">
-      <c r="B13" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="13" spans="2:26" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <f t="shared" si="1"/>
+        <v>87</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="2"/>
@@ -2986,16 +2814,16 @@
       <c r="K13">
         <v>25</v>
       </c>
-      <c r="P13" t="e" cm="1">
-        <f t="array" aca="1" ref="P13" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D13:O13),""""&amp;D13:O13&amp;"""",IF(D13:O13="",0,D13:O13)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P13" t="str" cm="1">
+        <f t="array" ref="P13">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D13:O13),""""&amp;D13:O13&amp;"""",IF(D13:O13="",0,D13:O13)))&amp;"],"</f>
+        <v>["machine",12,50,"Machine shop","REPAIR",0,0,25,0,0,0,0],</v>
       </c>
       <c r="S13" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} machine</v>
       </c>
     </row>
-    <row r="14" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C14" t="str">
         <f t="shared" si="2"/>
         <v>s</v>
@@ -3009,16 +2837,16 @@
       <c r="H14" t="s">
         <v>37</v>
       </c>
-      <c r="P14" t="e" cm="1">
-        <f t="array" aca="1" ref="P14" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D14:O14),""""&amp;D14:O14&amp;"""",IF(D14:O14="",0,D14:O14)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P14" t="str" cm="1">
+        <f t="array" ref="P14">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D14:O14),""""&amp;D14:O14&amp;"""",IF(D14:O14="",0,D14:O14)))&amp;"],"</f>
+        <v>["shuttle",0,0,"Shuttle bay","USE",0,0,0,0,0,0,0],</v>
       </c>
       <c r="S14" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} shuttle</v>
       </c>
     </row>
-    <row r="15" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C15" t="str">
         <f t="shared" si="2"/>
         <v>a</v>
@@ -3032,16 +2860,16 @@
       <c r="H15" t="s">
         <v>37</v>
       </c>
-      <c r="P15" t="e" cm="1">
-        <f t="array" aca="1" ref="P15" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D15:O15),""""&amp;D15:O15&amp;"""",IF(D15:O15="",0,D15:O15)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P15" t="str" cm="1">
+        <f t="array" ref="P15">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D15:O15),""""&amp;D15:O15&amp;"""",IF(D15:O15="",0,D15:O15)))&amp;"],"</f>
+        <v>["access",0,0,"Upgrade center","USE",0,0,0,0,0,0,0],</v>
       </c>
       <c r="S15" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} access</v>
       </c>
     </row>
-    <row r="16" spans="2:26" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:26" x14ac:dyDescent="0.3">
       <c r="C16" t="str">
         <f t="shared" si="2"/>
         <v>d</v>
@@ -3055,19 +2883,19 @@
       <c r="H16" t="s">
         <v>37</v>
       </c>
-      <c r="P16" t="e" cm="1">
-        <f t="array" aca="1" ref="P16" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D16:O16),""""&amp;D16:O16&amp;"""",IF(D16:O16="",0,D16:O16)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P16" t="str" cm="1">
+        <f t="array" ref="P16">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D16:O16),""""&amp;D16:O16&amp;"""",IF(D16:O16="",0,D16:O16)))&amp;"],"</f>
+        <v>["door",0,0,"ACCESS KEY NEEDED","USE",0,0,0,0,0,0,0],</v>
       </c>
       <c r="S16" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} door</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B17" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <f t="shared" si="1"/>
+        <v>100</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="2"/>
@@ -3097,19 +2925,19 @@
       <c r="N17">
         <v>5</v>
       </c>
-      <c r="P17" t="e" cm="1">
-        <f t="array" aca="1" ref="P17" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D17:O17),""""&amp;D17:O17&amp;"""",IF(D17:O17="",0,D17:O17)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P17" t="str" cm="1">
+        <f t="array" ref="P17">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D17:O17),""""&amp;D17:O17&amp;"""",IF(D17:O17="",0,D17:O17)))&amp;"],"</f>
+        <v>["mining",15,60,"Mining station","CAPTURE",10,0,0,0,10,5,0],</v>
       </c>
       <c r="S17" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} mining</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B18" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <f t="shared" si="1"/>
+        <v>75</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="2"/>
@@ -3136,19 +2964,19 @@
       <c r="N18">
         <v>10</v>
       </c>
-      <c r="P18" t="e" cm="1">
-        <f t="array" aca="1" ref="P18" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D18:O18),""""&amp;D18:O18&amp;"""",IF(D18:O18="",0,D18:O18)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P18" t="str" cm="1">
+        <f t="array" ref="P18">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D18:O18),""""&amp;D18:O18&amp;"""",IF(D18:O18="",0,D18:O18)))&amp;"],"</f>
+        <v>["scrapyard",10,40,"Scrapyard","CAPTURE",0,0,0,15,0,10,0],</v>
       </c>
       <c r="S18" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} scrapyard</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B19" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <f t="shared" si="1"/>
+        <v>127</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="2"/>
@@ -3181,19 +3009,19 @@
       <c r="O19">
         <v>5</v>
       </c>
-      <c r="P19" t="e" cm="1">
-        <f t="array" aca="1" ref="P19" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D19:O19),""""&amp;D19:O19&amp;"""",IF(D19:O19="",0,D19:O19)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P19" t="str" cm="1">
+        <f t="array" ref="P19">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D19:O19),""""&amp;D19:O19&amp;"""",IF(D19:O19="",0,D19:O19)))&amp;"],"</f>
+        <v>["data",12,70,"Data vault","CAPTURE",0,0,0,30,5,5,5],</v>
       </c>
       <c r="S19" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} data</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B20" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <f t="shared" si="1"/>
+        <v>125</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="2"/>
@@ -3223,19 +3051,19 @@
       <c r="O20">
         <v>5</v>
       </c>
-      <c r="P20" t="e" cm="1">
-        <f t="array" aca="1" ref="P20" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D20:O20),""""&amp;D20:O20&amp;"""",IF(D20:O20="",0,D20:O20)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P20" t="str" cm="1">
+        <f t="array" ref="P20">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D20:O20),""""&amp;D20:O20&amp;"""",IF(D20:O20="",0,D20:O20)))&amp;"],"</f>
+        <v>["supply",15,80,"Supply depot","CAPTURE",0,0,15,0,10,0,5],</v>
       </c>
       <c r="S20" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} supply</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B21" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f t="shared" si="1"/>
+        <v>140</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="2"/>
@@ -3265,19 +3093,19 @@
       <c r="O21">
         <v>10</v>
       </c>
-      <c r="P21" t="e" cm="1">
-        <f t="array" aca="1" ref="P21" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D21:O21),""""&amp;D21:O21&amp;"""",IF(D21:O21="",0,D21:O21)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P21" t="str" cm="1">
+        <f t="array" ref="P21">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D21:O21),""""&amp;D21:O21&amp;"""",IF(D21:O21="",0,D21:O21)))&amp;"],"</f>
+        <v>["fusion",10,90,"Fusion core","CAPTURE",20,0,0,0,0,10,10],</v>
       </c>
       <c r="S21" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} fusion</v>
       </c>
     </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B22" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <f t="shared" si="1"/>
+        <v>170</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="2"/>
@@ -3304,19 +3132,19 @@
       <c r="M22">
         <v>20</v>
       </c>
-      <c r="P22" t="e" cm="1">
-        <f t="array" aca="1" ref="P22" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D22:O22),""""&amp;D22:O22&amp;"""",IF(D22:O22="",0,D22:O22)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P22" t="str" cm="1">
+        <f t="array" ref="P22">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D22:O22),""""&amp;D22:O22&amp;"""",IF(D22:O22="",0,D22:O22)))&amp;"],"</f>
+        <v>["alloy",20,100,"Alloy plant","CAPTURE",30,0,0,0,20,0,0],</v>
       </c>
       <c r="S22" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} alloy</v>
       </c>
     </row>
-    <row r="23" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B23" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <f t="shared" si="1"/>
+        <v>127</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="2"/>
@@ -3346,16 +3174,16 @@
       <c r="O23">
         <v>5</v>
       </c>
-      <c r="P23" t="e" cm="1">
-        <f t="array" aca="1" ref="P23" ca="1">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D23:O23),""""&amp;D23:O23&amp;"""",IF(D23:O23="",0,D23:O23)))&amp;"],"</f>
-        <v>#NAME?</v>
+      <c r="P23" t="str" cm="1">
+        <f t="array" ref="P23">"["&amp;_xlfn.TEXTJOIN(",",FALSE,IF(ISTEXT(D23:O23),""""&amp;D23:O23&amp;"""",IF(D23:O23="",0,D23:O23)))&amp;"],"</f>
+        <v>["research",12,85,"Research lab","CAPTURE",10,0,0,0,0,15,5],</v>
       </c>
       <c r="S23" t="str">
         <f t="shared" si="3"/>
         <v xml:space="preserve"> * @property {number} research</v>
       </c>
     </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B24">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3365,7 +3193,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B25">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3375,7 +3203,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B26">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3385,7 +3213,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3395,7 +3223,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B28">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3405,7 +3233,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3415,7 +3243,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B30">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3425,7 +3253,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B31">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3436,14 +3264,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:AB2">
-    <cfRule type="duplicateValues" dxfId="27" priority="3"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C4:C31">
-    <cfRule type="duplicateValues" dxfId="26" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:AB2">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
deleted terminals somehow keep drawing
</commit_message>
<xml_diff>
--- a/docs/relay/design/scripting.xlsx
+++ b/docs/relay/design/scripting.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\js\games\docs\relay\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A73D56-4FBB-4BDF-8FDD-07529180D6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12580"/>
   </bookViews>
   <sheets>
     <sheet name="sheetwithani" sheetId="3" r:id="rId1"/>
     <sheet name="conventions" sheetId="4" r:id="rId2"/>
     <sheet name="bad" sheetId="1" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,14 +37,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -60,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="139">
   <si>
     <t>firstletter</t>
   </si>
@@ -453,12 +452,36 @@
   </si>
   <si>
     <t>req hazard on homebase only</t>
+  </si>
+  <si>
+    <t>smallenergy</t>
+  </si>
+  <si>
+    <t>smallwater</t>
+  </si>
+  <si>
+    <t>smallfood</t>
+  </si>
+  <si>
+    <t>smallparts</t>
+  </si>
+  <si>
+    <t>Small battery</t>
+  </si>
+  <si>
+    <t>Small water bottle</t>
+  </si>
+  <si>
+    <t>Small candy bar</t>
+  </si>
+  <si>
+    <t>Small circuits</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -980,26 +1003,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:T48"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.88671875" customWidth="1"/>
-    <col min="2" max="2" width="4.109375" customWidth="1"/>
+    <col min="1" max="1" width="1.90625" customWidth="1"/>
+    <col min="2" max="2" width="4.08984375" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="5.21875" customWidth="1"/>
+    <col min="4" max="4" width="5.1796875" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.77734375" customWidth="1"/>
-    <col min="8" max="15" width="7.109375" customWidth="1"/>
-    <col min="16" max="16" width="30.77734375" customWidth="1"/>
-    <col min="17" max="17" width="15.21875" customWidth="1"/>
-    <col min="18" max="18" width="12.21875" customWidth="1"/>
-    <col min="19" max="19" width="15.21875" customWidth="1"/>
-    <col min="20" max="20" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.36328125" customWidth="1"/>
+    <col min="7" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="15" width="7.08984375" customWidth="1"/>
+    <col min="16" max="16" width="30.81640625" customWidth="1"/>
+    <col min="17" max="17" width="15.1796875" customWidth="1"/>
+    <col min="18" max="18" width="12.1796875" customWidth="1"/>
+    <col min="19" max="19" width="15.1796875" customWidth="1"/>
+    <col min="20" max="20" width="15.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="H1" s="13" t="s">
         <v>60</v>
       </c>
@@ -1022,7 +1045,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>119</v>
       </c>
@@ -1062,7 +1085,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -1119,7 +1142,7 @@
         <v>['terminal','delay','bucket','pretty','action','energy','water','food','parts','antimatter','coolant','minerals','salvage','description','note','prereq'],</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="12" t="s">
         <v>65</v>
       </c>
@@ -1150,14 +1173,14 @@
         <v>71</v>
       </c>
       <c r="T4" t="str">
-        <f t="shared" ref="T4:T38" si="1">"["&amp;IF(ISNUMBER(C4),C4,IF(C4="",0,CHAR(39)&amp;C4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(D4),D4,IF(D4="",0,CHAR(39)&amp;D4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(E4),E4,IF(E4="",0,CHAR(39)&amp;E4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(F4),F4,IF(F4="",0,CHAR(39)&amp;F4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(G4),G4,IF(G4="",0,CHAR(39)&amp;G4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(H4),H4,IF(H4="",0,CHAR(39)&amp;H4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(I4),I4,IF(I4="",0,CHAR(39)&amp;I4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(J4),J4,IF(J4="",0,CHAR(39)&amp;J4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(K4),K4,IF(K4="",0,CHAR(39)&amp;K4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(L4),L4,IF(L4="",0,CHAR(39)&amp;L4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(M4),M4,IF(M4="",0,CHAR(39)&amp;M4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(N4),N4,IF(N4="",0,CHAR(39)&amp;N4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(O4),O4,IF(O4="",0,CHAR(39)&amp;O4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(P4),P4,IF(P4="",0,CHAR(39)&amp;P4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(Q4),Q4,IF(Q4="",0,CHAR(39)&amp;Q4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(R4),R4,IF(R4="",0,CHAR(39)&amp;R4&amp;CHAR(39)))&amp;"],"</f>
+        <f t="shared" ref="T4:T42" si="1">"["&amp;IF(ISNUMBER(C4),C4,IF(C4="",0,CHAR(39)&amp;C4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(D4),D4,IF(D4="",0,CHAR(39)&amp;D4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(E4),E4,IF(E4="",0,CHAR(39)&amp;E4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(F4),F4,IF(F4="",0,CHAR(39)&amp;F4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(G4),G4,IF(G4="",0,CHAR(39)&amp;G4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(H4),H4,IF(H4="",0,CHAR(39)&amp;H4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(I4),I4,IF(I4="",0,CHAR(39)&amp;I4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(J4),J4,IF(J4="",0,CHAR(39)&amp;J4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(K4),K4,IF(K4="",0,CHAR(39)&amp;K4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(L4),L4,IF(L4="",0,CHAR(39)&amp;L4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(M4),M4,IF(M4="",0,CHAR(39)&amp;M4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(N4),N4,IF(N4="",0,CHAR(39)&amp;N4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(O4),O4,IF(O4="",0,CHAR(39)&amp;O4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(P4),P4,IF(P4="",0,CHAR(39)&amp;P4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(Q4),Q4,IF(Q4="",0,CHAR(39)&amp;Q4&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(R4),R4,IF(R4="",0,CHAR(39)&amp;R4&amp;CHAR(39)))&amp;"],"</f>
         <v>['reactor',15,0,'Reactor','REPAIR',50,0,0,0,0,0,0,0,0,'base',0],</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="12"/>
       <c r="B5">
-        <f t="shared" ref="B5:B44" si="2">SUM(H5:O5)</f>
+        <f t="shared" ref="B5:B48" si="2">SUM(H5:O5)</f>
         <v>30</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1190,7 +1213,7 @@
         <v>['solar',8,10,'Solar Array','REPAIR',30,0,0,0,0,0,0,0,0,'upgrade1','reactor'],</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="12"/>
       <c r="B6">
         <f t="shared" si="2"/>
@@ -1226,7 +1249,7 @@
         <v>['life',12,0,'Life Support','REPAIR',0,20,20,0,0,0,0,0,0,'base',0],</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="12"/>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -1262,7 +1285,7 @@
         <v>['water',6,10,'Water Recycler','REPAIR',0,30,0,0,0,0,0,0,0,'upgrade1','life'],</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="12"/>
       <c r="B8">
         <f t="shared" si="2"/>
@@ -1298,7 +1321,7 @@
         <v>['hydro',13,10,'Hydroponics','REPAIR',0,0,30,0,0,0,0,0,0,'upgrade1','life'],</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="12"/>
       <c r="B9">
         <f t="shared" si="2"/>
@@ -1331,7 +1354,7 @@
         <v>['cargo',4,0,'Cargo bay','REPAIR',0,0,0,20,0,0,0,0,0,'base',0],</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="12"/>
       <c r="B10">
         <f t="shared" si="2"/>
@@ -1367,7 +1390,7 @@
         <v>['comms',11,10,'Comms array','REPAIR',0,0,0,50,0,0,0,0,0,'upgrade1','cargo'],</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="12"/>
       <c r="B11">
         <f t="shared" si="2"/>
@@ -1403,7 +1426,7 @@
         <v>['fab',13,20,'Fabricator','REPAIR',0,0,0,10,0,0,0,0,0,'upgrade2','comms'],</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="12"/>
       <c r="B12">
         <f t="shared" si="2"/>
@@ -1442,7 +1465,7 @@
         <v>['med',14,20,'Medical bay','REPAIR',0,10,10,0,0,0,0,0,0,'upgrade2','water,hydro'],</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="12"/>
       <c r="B13">
         <f t="shared" si="2"/>
@@ -1481,7 +1504,7 @@
         <v>['anti',20,20,'Antimatter Chamber','REPAIR',10,0,0,0,5,0,0,0,0,'upgrade2','solar'],</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>66</v>
       </c>
@@ -1515,7 +1538,7 @@
         <v>['hazard',0,30,'Space Hazard Unit','REPAIR',0,0,0,0,0,0,0,0,'Allows you to explore space.','upgrade3','fab,med,anti'],</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" s="15"/>
       <c r="B15">
         <f t="shared" si="2"/>
@@ -1539,7 +1562,7 @@
         <v>['obs',0,0,'Observatory','WORLDMAP',0,0,0,0,0,0,0,0,'Lets you peek into the endless void of space.',0,0],</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="15"/>
       <c r="B16">
         <f t="shared" si="2"/>
@@ -1565,7 +1588,7 @@
         <v>['shuttle',0,0,'Shuttle bay','TRAVEL',0,0,0,0,0,0,0,0,'Travel to new locations!','req hazard on homebase only',0],</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="15"/>
       <c r="B17">
         <f t="shared" si="2"/>
@@ -1589,7 +1612,7 @@
         <v>['upgrade',0,0,'Upgrade center','SEEUPGRADES',0,0,0,0,0,0,0,0,'See available upgrades.',0,0],</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
         <v>67</v>
       </c>
@@ -1622,7 +1645,7 @@
         <v>['mining',5,30,'Mining station','CAPTURE',0,0,0,0,0,0,15,0,0,0,0],</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19">
         <f t="shared" si="2"/>
@@ -1653,7 +1676,7 @@
         <v>['scrapyard',5,30,'Scrapyard','CAPTURE',0,0,0,0,0,0,0,15,0,0,0],</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="14"/>
       <c r="B20">
         <f t="shared" si="2"/>
@@ -1690,7 +1713,7 @@
         <v>['data',5,30,'Data vault','CAPTURE',0,0,0,0,0,5,5,5,0,0,0],</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" s="14"/>
       <c r="B21">
         <f t="shared" si="2"/>
@@ -1718,7 +1741,7 @@
         <v>['supply',5,30,'Supply depot','CAPTURE',0,0,0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" s="14"/>
       <c r="B22">
         <f t="shared" si="2"/>
@@ -1749,7 +1772,7 @@
         <v>['fusion',5,40,'Fusion core','CAPTURE',0,0,0,0,15,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" s="14"/>
       <c r="B23">
         <f t="shared" si="2"/>
@@ -1783,7 +1806,7 @@
         <v>['alloy',5,30,'Alloy plant','CAPTURE',0,0,0,0,0,0,10,5,0,0,0],</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="14"/>
       <c r="B24">
         <f t="shared" si="2"/>
@@ -1820,7 +1843,7 @@
         <v>['research',5,40,'Research lab','CAPTURE',0,0,0,0,5,5,0,5,0,0,0],</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" s="14"/>
       <c r="B25">
         <f t="shared" si="2"/>
@@ -1848,7 +1871,7 @@
         <v>['chestenergy',0,20,'Energy cells','CLAIM',120,0,0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26" s="14"/>
       <c r="B26">
         <f t="shared" si="2"/>
@@ -1876,7 +1899,7 @@
         <v>['chestwater',0,20,'Ice blocks','CLAIM',0,120,0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="14"/>
       <c r="B27">
         <f t="shared" si="2"/>
@@ -1904,7 +1927,7 @@
         <v>['chestfood',0,20,'Nutrient packs','CLAIM',0,0,120,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" s="14"/>
       <c r="B28">
         <f t="shared" si="2"/>
@@ -1932,340 +1955,380 @@
         <v>['chestparts',0,20,'Parts box','CLAIM',0,0,0,120,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" s="14"/>
       <c r="B29">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="E29">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="G29" t="s">
         <v>86</v>
       </c>
-      <c r="L29">
-        <v>80</v>
+      <c r="H29">
+        <v>10</v>
       </c>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="T29" t="str">
         <f t="shared" si="1"/>
-        <v>['chestantimatter',0,40,'Antimatter traces','CLAIM',0,0,0,0,80,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['smallenergy',0,0,'Small battery','CLAIM',10,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" s="14"/>
       <c r="B30">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
       <c r="E30">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="G30" t="s">
         <v>86</v>
       </c>
-      <c r="M30">
-        <v>80</v>
+      <c r="I30">
+        <v>10</v>
       </c>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
       <c r="T30" t="str">
         <f t="shared" si="1"/>
-        <v>['chestcoolant',0,40,'Coolant remains','CLAIM',0,0,0,0,0,80,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['smallwater',0,0,'Small water bottle','CLAIM',0,10,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="14"/>
       <c r="B31">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>82</v>
+        <v>133</v>
       </c>
       <c r="E31">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="G31" t="s">
         <v>86</v>
       </c>
-      <c r="N31">
-        <v>80</v>
+      <c r="J31">
+        <v>10</v>
       </c>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
       <c r="T31" t="str">
         <f t="shared" si="1"/>
-        <v>['chestmineral',0,40,'Mineral residue','CLAIM',0,0,0,0,0,0,80,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['smallfood',0,0,'Small candy bar','CLAIM',0,0,10,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="E32">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>89</v>
+        <v>138</v>
       </c>
       <c r="G32" t="s">
         <v>86</v>
       </c>
-      <c r="O32">
-        <v>80</v>
+      <c r="K32">
+        <v>10</v>
       </c>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
       <c r="T32" t="str">
         <f t="shared" si="1"/>
-        <v>['chestsalvage',0,40,'Salvage pack','CLAIM',0,0,0,0,0,0,0,80,0,0,0],</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['smallparts',0,0,'Small circuits','CLAIM',0,0,0,10,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" s="14"/>
       <c r="B33">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G33" t="s">
-        <v>107</v>
+        <v>86</v>
+      </c>
+      <c r="L33">
+        <v>80</v>
       </c>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
       <c r="T33" t="str">
         <f t="shared" si="1"/>
-        <v>['door_easy',0,0,'Damaged door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['chestantimatter',0,40,'Antimatter traces','CLAIM',0,0,0,0,80,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A34" s="14"/>
       <c r="B34">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="E34">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G34" t="s">
-        <v>107</v>
+        <v>86</v>
+      </c>
+      <c r="M34">
+        <v>80</v>
       </c>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
       <c r="T34" t="str">
         <f t="shared" si="1"/>
-        <v>['door_medium',0,20,'Locked door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['chestcoolant',0,40,'Coolant remains','CLAIM',0,0,0,0,0,80,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35" s="14"/>
       <c r="B35">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
       <c r="E35">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>125</v>
+        <v>87</v>
       </c>
       <c r="G35" t="s">
-        <v>107</v>
+        <v>86</v>
+      </c>
+      <c r="N35">
+        <v>80</v>
       </c>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
       <c r="T35" t="str">
         <f t="shared" si="1"/>
-        <v>['door_hard',0,50,'Reinforced door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+        <v>['chestmineral',0,40,'Mineral residue','CLAIM',0,0,0,0,0,0,80,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36" s="14"/>
       <c r="B36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>124</v>
+        <v>84</v>
       </c>
       <c r="E36">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>112</v>
+        <v>89</v>
+      </c>
+      <c r="G36" t="s">
+        <v>86</v>
+      </c>
+      <c r="O36">
+        <v>80</v>
       </c>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
       <c r="T36" t="str">
         <f t="shared" si="1"/>
+        <v>['chestsalvage',0,40,'Salvage pack','CLAIM',0,0,0,0,0,0,0,80,0,0,0],</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A37" s="14"/>
+      <c r="B37">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G37" t="s">
+        <v>107</v>
+      </c>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+      <c r="T37" t="str">
+        <f t="shared" si="1"/>
+        <v>['door_easy',0,0,'Damaged door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A38" s="14"/>
+      <c r="B38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E38">
+        <v>20</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G38" t="s">
+        <v>107</v>
+      </c>
+      <c r="P38" s="3"/>
+      <c r="Q38" s="3"/>
+      <c r="T38" t="str">
+        <f t="shared" si="1"/>
+        <v>['door_medium',0,20,'Locked door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A39" s="14"/>
+      <c r="B39">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39">
+        <v>50</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G39" t="s">
+        <v>107</v>
+      </c>
+      <c r="P39" s="3"/>
+      <c r="Q39" s="3"/>
+      <c r="T39" t="str">
+        <f t="shared" si="1"/>
+        <v>['door_hard',0,50,'Reinforced door','HACK',0,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A40" s="14"/>
+      <c r="B40">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E40">
+        <v>70</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="P40" s="3"/>
+      <c r="Q40" s="3"/>
+      <c r="T40" t="str">
+        <f t="shared" si="1"/>
         <v>['door_extreme',0,70,'High security door',0,0,0,0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="C37" s="9" t="s">
+      <c r="B41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E37">
-        <v>10</v>
-      </c>
-      <c r="F37" s="9" t="s">
+      <c r="E41">
+        <v>10</v>
+      </c>
+      <c r="F41" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G37" t="s">
-        <v>108</v>
-      </c>
-      <c r="P37" s="9"/>
-      <c r="Q37" s="9"/>
-      <c r="T37" t="str">
-        <f t="shared" si="1"/>
-        <v>['plants',0,10,'Plants','RESTORE',0,0,0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A38" s="12"/>
-      <c r="B38">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="E38">
-        <v>10</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" t="s">
-        <v>108</v>
-      </c>
-      <c r="P38" s="9"/>
-      <c r="Q38" s="9"/>
-      <c r="T38" t="str">
-        <f t="shared" si="1"/>
-        <v>['fridge',0,10,'Fridge','RESTORE',0,0,0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="C39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" t="s">
-        <v>108</v>
-      </c>
-      <c r="P39" s="9"/>
-      <c r="Q39" s="9"/>
-      <c r="T39" t="str">
-        <f t="shared" ref="T39:T44" si="3">"["&amp;IF(ISNUMBER(C39),C39,IF(C39="",0,CHAR(39)&amp;C39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(D39),D39,IF(D39="",0,CHAR(39)&amp;D39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(E39),E39,IF(E39="",0,CHAR(39)&amp;E39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(F39),F39,IF(F39="",0,CHAR(39)&amp;F39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(G39),G39,IF(G39="",0,CHAR(39)&amp;G39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(H39),H39,IF(H39="",0,CHAR(39)&amp;H39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(I39),I39,IF(I39="",0,CHAR(39)&amp;I39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(J39),J39,IF(J39="",0,CHAR(39)&amp;J39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(K39),K39,IF(K39="",0,CHAR(39)&amp;K39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(L39),L39,IF(L39="",0,CHAR(39)&amp;L39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(M39),M39,IF(M39="",0,CHAR(39)&amp;M39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(N39),N39,IF(N39="",0,CHAR(39)&amp;N39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(O39),O39,IF(O39="",0,CHAR(39)&amp;O39&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(P39),P39,IF(P39="",0,CHAR(39)&amp;P39&amp;CHAR(39)))&amp;"],"</f>
-        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A40" s="12"/>
-      <c r="B40">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="C40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" t="s">
-        <v>108</v>
-      </c>
-      <c r="P40" s="9"/>
-      <c r="Q40" s="9"/>
-      <c r="T40" t="str">
-        <f t="shared" si="3"/>
-        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A41" s="12"/>
-      <c r="B41">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="C41" s="9"/>
-      <c r="F41" s="9"/>
       <c r="G41" t="s">
         <v>108</v>
       </c>
       <c r="P41" s="9"/>
       <c r="Q41" s="9"/>
       <c r="T41" t="str">
-        <f t="shared" si="3"/>
-        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="shared" si="1"/>
+        <v>['plants',0,10,'Plants','RESTORE',0,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" s="12"/>
       <c r="B42">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C42" s="9"/>
-      <c r="F42" s="9"/>
+      <c r="C42" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E42">
+        <v>10</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>110</v>
+      </c>
       <c r="G42" t="s">
         <v>108</v>
       </c>
       <c r="P42" s="9"/>
       <c r="Q42" s="9"/>
       <c r="T42" t="str">
-        <f t="shared" si="3"/>
-        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="shared" si="1"/>
+        <v>['fridge',0,10,'Fridge','RESTORE',0,0,0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A43" s="12"/>
       <c r="B43">
         <f t="shared" si="2"/>
@@ -2279,11 +2342,11 @@
       <c r="P43" s="9"/>
       <c r="Q43" s="9"/>
       <c r="T43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="T43:T48" si="3">"["&amp;IF(ISNUMBER(C43),C43,IF(C43="",0,CHAR(39)&amp;C43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(D43),D43,IF(D43="",0,CHAR(39)&amp;D43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(E43),E43,IF(E43="",0,CHAR(39)&amp;E43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(F43),F43,IF(F43="",0,CHAR(39)&amp;F43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(G43),G43,IF(G43="",0,CHAR(39)&amp;G43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(H43),H43,IF(H43="",0,CHAR(39)&amp;H43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(I43),I43,IF(I43="",0,CHAR(39)&amp;I43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(J43),J43,IF(J43="",0,CHAR(39)&amp;J43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(K43),K43,IF(K43="",0,CHAR(39)&amp;K43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(L43),L43,IF(L43="",0,CHAR(39)&amp;L43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(M43),M43,IF(M43="",0,CHAR(39)&amp;M43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(N43),N43,IF(N43="",0,CHAR(39)&amp;N43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(O43),O43,IF(O43="",0,CHAR(39)&amp;O43&amp;CHAR(39)))&amp;","&amp;IF(ISNUMBER(P43),P43,IF(P43="",0,CHAR(39)&amp;P43&amp;CHAR(39)))&amp;"],"</f>
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44" s="12"/>
       <c r="B44">
         <f t="shared" si="2"/>
@@ -2301,16 +2364,88 @@
         <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
       </c>
     </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A45" s="12"/>
+      <c r="B45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" t="s">
+        <v>108</v>
+      </c>
+      <c r="P45" s="9"/>
+      <c r="Q45" s="9"/>
+      <c r="T45" t="str">
+        <f t="shared" si="3"/>
+        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A46" s="12"/>
+      <c r="B46">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" t="s">
+        <v>108</v>
+      </c>
+      <c r="P46" s="9"/>
+      <c r="Q46" s="9"/>
+      <c r="T46" t="str">
+        <f t="shared" si="3"/>
+        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A47" s="12"/>
+      <c r="B47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" t="s">
+        <v>108</v>
+      </c>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="9"/>
+      <c r="T47" t="str">
+        <f t="shared" si="3"/>
+        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A48" s="12"/>
+      <c r="B48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="C48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" t="s">
+        <v>108</v>
+      </c>
+      <c r="P48" s="9"/>
+      <c r="Q48" s="9"/>
+      <c r="T48" t="str">
+        <f t="shared" si="3"/>
+        <v>[0,0,0,0,'RESTORE',0,0,0,0,0,0,0,0,0],</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A37:A44"/>
+    <mergeCell ref="A41:A48"/>
     <mergeCell ref="H1:K1"/>
     <mergeCell ref="A4:A13"/>
-    <mergeCell ref="A18:A36"/>
+    <mergeCell ref="A18:A40"/>
     <mergeCell ref="L1:O1"/>
     <mergeCell ref="A14:A17"/>
   </mergeCells>
-  <conditionalFormatting sqref="C1:C17 C37:C1048576">
+  <conditionalFormatting sqref="C41:C1048576 C1:C17">
     <cfRule type="duplicateValues" dxfId="11" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
@@ -2319,7 +2454,7 @@
   <conditionalFormatting sqref="D2:O2 T2:U2">
     <cfRule type="duplicateValues" dxfId="9" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E4:E62">
+  <conditionalFormatting sqref="E4:E66">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2331,7 +2466,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F37:F44">
+  <conditionalFormatting sqref="F41:F48">
     <cfRule type="duplicateValues" dxfId="8" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2">
@@ -2340,7 +2475,7 @@
   <conditionalFormatting sqref="P3">
     <cfRule type="duplicateValues" dxfId="6" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P37:Q44">
+  <conditionalFormatting sqref="P41:Q48">
     <cfRule type="duplicateValues" dxfId="5" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3:R3">
@@ -2355,19 +2490,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="97.44140625" defaultRowHeight="57" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="97.453125" defaultRowHeight="57" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="97.44140625" style="10"/>
+    <col min="1" max="16384" width="97.453125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>120</v>
       </c>
@@ -2378,17 +2513,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:Z31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="6" width="7.33203125" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="5" max="6" width="7.36328125" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:26" x14ac:dyDescent="0.35">
       <c r="D2" t="s">
         <v>0</v>
       </c>
@@ -2460,7 +2595,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -2508,7 +2643,7 @@
         <v>["terminal","delay","question","pretty","action","energy","food","water","parts","metals","titanium","alloy"],</v>
       </c>
     </row>
-    <row r="4" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B4">
         <f>SUM(E4:AA4)</f>
         <v>55</v>
@@ -2540,7 +2675,7 @@
         <v>["reactor",15,0,"Reactor","REPAIR",40,0,0,0,0,0,0],</v>
       </c>
     </row>
-    <row r="5" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B5">
         <f t="shared" ref="B5:B31" si="1">SUM(E5:AA5)</f>
         <v>55</v>
@@ -2576,7 +2711,7 @@
         <v xml:space="preserve"> * @property {number} solar</v>
       </c>
     </row>
-    <row r="6" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B6">
         <f t="shared" si="1"/>
         <v>57</v>
@@ -2615,7 +2750,7 @@
         <v xml:space="preserve"> * @property {number} hydro</v>
       </c>
     </row>
-    <row r="7" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B7">
         <f t="shared" si="1"/>
         <v>55</v>
@@ -2651,7 +2786,7 @@
         <v xml:space="preserve"> * @property {number} water</v>
       </c>
     </row>
-    <row r="8" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B8">
         <f t="shared" si="1"/>
         <v>48</v>
@@ -2690,7 +2825,7 @@
         <v xml:space="preserve"> * @property {number} cargo</v>
       </c>
     </row>
-    <row r="9" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B9">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -2726,7 +2861,7 @@
         <v xml:space="preserve"> * @property {number} comms</v>
       </c>
     </row>
-    <row r="10" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B10">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -2765,7 +2900,7 @@
         <v xml:space="preserve"> * @property {number} fab</v>
       </c>
     </row>
-    <row r="11" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B11">
         <f t="shared" si="1"/>
         <v>50</v>
@@ -2801,7 +2936,7 @@
         <v xml:space="preserve"> * @property {number} med</v>
       </c>
     </row>
-    <row r="12" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B12">
         <f t="shared" si="1"/>
         <v>55</v>
@@ -2840,7 +2975,7 @@
         <v xml:space="preserve"> * @property {number} life</v>
       </c>
     </row>
-    <row r="13" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:26" x14ac:dyDescent="0.35">
       <c r="B13">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -2876,7 +3011,7 @@
         <v xml:space="preserve"> * @property {number} machine</v>
       </c>
     </row>
-    <row r="14" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:26" x14ac:dyDescent="0.35">
       <c r="C14" t="str">
         <f t="shared" si="2"/>
         <v>s</v>
@@ -2899,7 +3034,7 @@
         <v xml:space="preserve"> * @property {number} shuttle</v>
       </c>
     </row>
-    <row r="15" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:26" x14ac:dyDescent="0.35">
       <c r="C15" t="str">
         <f t="shared" si="2"/>
         <v>a</v>
@@ -2922,7 +3057,7 @@
         <v xml:space="preserve"> * @property {number} access</v>
       </c>
     </row>
-    <row r="16" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:26" x14ac:dyDescent="0.35">
       <c r="C16" t="str">
         <f t="shared" si="2"/>
         <v>d</v>
@@ -2945,7 +3080,7 @@
         <v xml:space="preserve"> * @property {number} door</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B17">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -2987,7 +3122,7 @@
         <v xml:space="preserve"> * @property {number} mining</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B18">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -3026,7 +3161,7 @@
         <v xml:space="preserve"> * @property {number} scrapyard</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B19">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -3071,7 +3206,7 @@
         <v xml:space="preserve"> * @property {number} data</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B20">
         <f t="shared" si="1"/>
         <v>125</v>
@@ -3113,7 +3248,7 @@
         <v xml:space="preserve"> * @property {number} supply</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B21">
         <f t="shared" si="1"/>
         <v>140</v>
@@ -3155,7 +3290,7 @@
         <v xml:space="preserve"> * @property {number} fusion</v>
       </c>
     </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B22">
         <f t="shared" si="1"/>
         <v>170</v>
@@ -3194,7 +3329,7 @@
         <v xml:space="preserve"> * @property {number} alloy</v>
       </c>
     </row>
-    <row r="23" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B23">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -3236,7 +3371,7 @@
         <v xml:space="preserve"> * @property {number} research</v>
       </c>
     </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B24">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3246,7 +3381,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B25">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3256,7 +3391,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B26">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3266,7 +3401,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3276,7 +3411,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B28">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3286,7 +3421,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3296,7 +3431,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B30">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3306,7 +3441,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B31">
         <f t="shared" si="1"/>
         <v>0</v>

</xml_diff>